<commit_message>
Use original activity columns in participation tracker
</commit_message>
<xml_diff>
--- a/docs/05-team-management/team-tracker.xlsx
+++ b/docs/05-team-management/team-tracker.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Participation" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Participation'!$A$1:$H$10</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Participation'!$A$1:$N$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -96,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -119,6 +119,12 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -197,17 +203,23 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TeamParticipation" displayName="TeamParticipation" ref="A4:H10" headerRowCount="1">
-  <autoFilter ref="A4:H10"/>
-  <tableColumns count="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TeamParticipation" displayName="TeamParticipation" ref="A4:N10" headerRowCount="1">
+  <autoFilter ref="A4:N10"/>
+  <tableColumns count="14">
     <tableColumn id="1" name="Team Member"/>
-    <tableColumn id="2" name="Week 3"/>
-    <tableColumn id="3" name="Week 4"/>
-    <tableColumn id="4" name="Week 5"/>
-    <tableColumn id="5" name="Week 6"/>
-    <tableColumn id="6" name="Week 7"/>
-    <tableColumn id="7" name="Week 8"/>
-    <tableColumn id="8" name="Week 9"/>
+    <tableColumn id="2" name="Sep 3 - In-Class Activity: TPS Workflow"/>
+    <tableColumn id="3" name="Sep 5 - Out-of-Class: GitHub Setup"/>
+    <tableColumn id="4" name="Sep 8 - Milestone 1: Proposal"/>
+    <tableColumn id="5" name="Sep 10 - Live Build: HTML Structure"/>
+    <tableColumn id="6" name="Sep 13 - Milestone 1"/>
+    <tableColumn id="7" name="Sep 20 - Week 3 Group Exercise Pack"/>
+    <tableColumn id="8" name="Week 4 Group Exercise"/>
+    <tableColumn id="9" name="Sept 26 - Week 5 Group Exercise"/>
+    <tableColumn id="10" name="October 7 - Week 6 Group Exercise"/>
+    <tableColumn id="11" name="October 11 - Week 7 Group Exercise"/>
+    <tableColumn id="12" name="October 18 - Milestone 2"/>
+    <tableColumn id="13" name="October 18 - Week 8 Group Exercise"/>
+    <tableColumn id="14" name="October 25 - Week 9 Group Exercise"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -502,17 +514,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -530,45 +548,75 @@
       </c>
     </row>
     <row r="3" ht="10" customHeight="1"/>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="4" ht="78" customHeight="1">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>Team Member</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Week 3</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Week 4</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Week 5</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Week 6</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>Week 7</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>Week 8</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>Week 9</t>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Sep 3 - In-Class Activity: TPS Workflow</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>Sep 5 - Out-of-Class: GitHub Setup</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>Sep 8 - Milestone 1: Proposal</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>Sep 10 - Live Build: HTML Structure</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>Sep 13 - Milestone 1</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Sep 20 - Week 3 Group Exercise Pack</t>
+        </is>
+      </c>
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>Week 4 Group Exercise</t>
+        </is>
+      </c>
+      <c r="I4" s="10" t="inlineStr">
+        <is>
+          <t>Sept 26 - Week 5 Group Exercise</t>
+        </is>
+      </c>
+      <c r="J4" s="10" t="inlineStr">
+        <is>
+          <t>October 7 - Week 6 Group Exercise</t>
+        </is>
+      </c>
+      <c r="K4" s="10" t="inlineStr">
+        <is>
+          <t>October 11 - Week 7 Group Exercise</t>
+        </is>
+      </c>
+      <c r="L4" s="10" t="inlineStr">
+        <is>
+          <t>October 18 - Milestone 2</t>
+        </is>
+      </c>
+      <c r="M4" s="10" t="inlineStr">
+        <is>
+          <t>October 18 - Week 8 Group Exercise</t>
+        </is>
+      </c>
+      <c r="N4" s="10" t="inlineStr">
+        <is>
+          <t>October 25 - Week 9 Group Exercise</t>
         </is>
       </c>
     </row>
@@ -599,6 +647,24 @@
       <c r="H5" s="6" t="n">
         <v>100</v>
       </c>
+      <c r="I5" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
@@ -627,6 +693,24 @@
       <c r="H6" s="8" t="n">
         <v>100</v>
       </c>
+      <c r="I6" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="J6" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="K6" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="L6" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="M6" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="N6" s="8" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
@@ -655,6 +739,24 @@
       <c r="H7" s="6" t="n">
         <v>100</v>
       </c>
+      <c r="I7" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="L7" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="M7" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="N7" s="6" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
@@ -683,6 +785,24 @@
       <c r="H8" s="8" t="n">
         <v>100</v>
       </c>
+      <c r="I8" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="J8" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="K8" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="L8" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="M8" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="N8" s="8" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
@@ -711,6 +831,24 @@
       <c r="H9" s="6" t="n">
         <v>100</v>
       </c>
+      <c r="I9" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="J9" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="K9" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="L9" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="M9" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="N9" s="6" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
@@ -739,11 +877,29 @@
       <c r="H10" s="8" t="n">
         <v>100</v>
       </c>
+      <c r="I10" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="J10" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="K10" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="L10" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="M10" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="N10" s="8" t="n">
+        <v>100</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.35" right="0.35" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>

</xml_diff>